<commit_message>
Lab pig slurry tests added
</commit_message>
<xml_diff>
--- a/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-soil-data.xlsx
+++ b/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-soil-data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-trails\2026-01-06-cattle-slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799BE4A7-7988-43F5-B094-49B235358EED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9564C682-2A05-461C-84B5-5E8E0EAF5FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pH" sheetId="1" r:id="rId1"/>
@@ -514,7 +514,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A9324FE-FEE3-4E64-AF93-D2D362EC8B69}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
@@ -652,99 +652,99 @@
         <v>23</v>
       </c>
     </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="2">
+        <v>4.2699999999999996</v>
+      </c>
+      <c r="E8">
+        <v>72.462999999999994</v>
+      </c>
+      <c r="F8">
+        <v>61.975999999999999</v>
+      </c>
+      <c r="G8">
+        <f>F8-D8</f>
+        <v>57.706000000000003</v>
+      </c>
+      <c r="H8">
+        <f>E8-F8</f>
+        <v>10.486999999999995</v>
+      </c>
+      <c r="I8" s="3">
+        <f>H8/G8</f>
+        <v>0.18173153571552342</v>
+      </c>
+    </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="2">
-        <v>4.2699999999999996</v>
+        <v>17</v>
+      </c>
+      <c r="D9">
+        <v>4.2729999999999997</v>
       </c>
       <c r="E9">
-        <v>72.462999999999994</v>
+        <v>64.980999999999995</v>
       </c>
       <c r="F9">
-        <v>61.975999999999999</v>
+        <v>55.631999999999998</v>
       </c>
       <c r="G9">
         <f>F9-D9</f>
-        <v>57.706000000000003</v>
+        <v>51.358999999999995</v>
       </c>
       <c r="H9">
         <f>E9-F9</f>
-        <v>10.486999999999995</v>
+        <v>9.3489999999999966</v>
       </c>
       <c r="I9" s="3">
         <f>H9/G9</f>
-        <v>0.18173153571552342</v>
+        <v>0.18203236044315499</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D10">
         <v>4.2729999999999997</v>
       </c>
       <c r="E10">
-        <v>64.980999999999995</v>
+        <v>56.356000000000002</v>
       </c>
       <c r="F10">
-        <v>55.631999999999998</v>
+        <v>48.308</v>
       </c>
       <c r="G10">
         <f>F10-D10</f>
-        <v>51.358999999999995</v>
+        <v>44.034999999999997</v>
       </c>
       <c r="H10">
         <f>E10-F10</f>
-        <v>9.3489999999999966</v>
+        <v>8.0480000000000018</v>
       </c>
       <c r="I10" s="3">
         <f>H10/G10</f>
-        <v>0.18203236044315499</v>
+        <v>0.1827637106846827</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11">
-        <v>4.2729999999999997</v>
-      </c>
-      <c r="E11">
-        <v>56.356000000000002</v>
-      </c>
-      <c r="F11">
-        <v>48.308</v>
-      </c>
-      <c r="G11">
-        <f>F11-D11</f>
-        <v>44.034999999999997</v>
-      </c>
-      <c r="H11">
-        <f>E11-F11</f>
-        <v>8.0480000000000018</v>
-      </c>
       <c r="I11" s="3">
-        <f>H11/G11</f>
-        <v>0.1827637106846827</v>
+        <f>AVERAGE(I8:I10)</f>
+        <v>0.18217586894778703</v>
+      </c>
+      <c r="J11" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="I12" s="3">
-        <f>AVERAGE(I9:I11)</f>
-        <v>0.18217586894778703</v>
+        <f>_xlfn.STDEV.P(I8:I10)</f>
+        <v>4.3342997121106203E-4</v>
       </c>
       <c r="J12" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="I13" s="3">
-        <f>_xlfn.STDEV.P(I9:I11)</f>
-        <v>4.3342997121106203E-4</v>
-      </c>
-      <c r="J13" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>